<commit_message>
Mark reviewed Part C labels high confidence
</commit_message>
<xml_diff>
--- a/data/annotations/part_c/DJI_20260107143259_0005_surface_cover_annotations.xlsx
+++ b/data/annotations/part_c/DJI_20260107143259_0005_surface_cover_annotations.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -5788,7 +5788,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">

</xml_diff>